<commit_message>
Second commit of MyORangeHRM Project
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10713"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HITENDRA VERMA\eclipse-workspace\OrangeHRMProject\src\test\resources\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/apm759/IdeaProjects/OrangeHRMProject/src/test/resources/testdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F9A4959-960F-45B2-9C3D-D28E0B95F543}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C8F69BA-C983-A947-BE7C-E6F0821F0403}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="validLoginData" sheetId="1" r:id="rId1"/>
@@ -383,9 +383,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -393,7 +393,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -412,9 +412,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F80A6D2-5586-454F-9399-C264D9CD4478}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -422,7 +422,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -438,12 +438,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7BDAB81-8119-4FF4-8BA6-76B8C63FA556}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="11.1796875" customWidth="1"/>
+    <col min="2" max="2" width="11.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -451,7 +451,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>

</xml_diff>